<commit_message>
ajustes para asegurados vigentes y analisis de polizas
</commit_message>
<xml_diff>
--- a/EXCEL UTILITARIOS/CALCULO  VISUALTIME - SALUD V2.xlsx
+++ b/EXCEL UTILITARIOS/CALCULO  VISUALTIME - SALUD V2.xlsx
@@ -8,9 +8,9 @@
       <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="C:\D\DATOS TRABAJO\NUEVO CORE\ORACLE_SQL\EXCEL UTILITARIOS\"/>
     </mc:Choice>
   </mc:AlternateContent>
-  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{00F437D4-2815-4688-A678-FD5778EA3203}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
+  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{010BF96A-8715-4F89-9B5C-E79EE5ECEEE2}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
   <bookViews>
-    <workbookView xWindow="-108" yWindow="-108" windowWidth="23256" windowHeight="13896" tabRatio="751" activeTab="2" xr2:uid="{00000000-000D-0000-FFFF-FFFF00000000}"/>
+    <workbookView xWindow="28680" yWindow="-120" windowWidth="20730" windowHeight="11040" tabRatio="751" activeTab="2" xr2:uid="{00000000-000D-0000-FFFF-FFFF00000000}"/>
   </bookViews>
   <sheets>
     <sheet name="FRECUENCIAS" sheetId="18" r:id="rId1"/>
@@ -2474,7 +2474,7 @@
         <v>42</v>
       </c>
       <c r="F2" s="115">
-        <v>1</v>
+        <v>2</v>
       </c>
       <c r="G2" s="116"/>
       <c r="H2" s="117"/>
@@ -2538,7 +2538,8 @@
       </c>
       <c r="E4" s="108"/>
       <c r="F4" s="98">
-        <v>620.91288999999995</v>
+        <f>2819.87+2387.808</f>
+        <v>5207.6779999999999</v>
       </c>
       <c r="G4" s="99">
         <v>0</v>
@@ -2548,11 +2549,11 @@
       </c>
       <c r="I4" s="94">
         <f>IF(B4="SI",IF($D4="SI",($F4+$G4+$H4) / (1- SUM($D$16:$D$20)),$F4),0)</f>
-        <v>796.04216666666662</v>
+        <v>6676.5102564102563</v>
       </c>
       <c r="J4" s="149">
         <f>$K$3*$I4</f>
-        <v>69.828022817833329</v>
+        <v>585.65680318205125</v>
       </c>
       <c r="L4" s="10"/>
     </row>
@@ -2568,17 +2569,17 @@
       </c>
       <c r="E5" s="92"/>
       <c r="F5" s="100">
-        <v>0</v>
+        <v>1185.5332000000001</v>
       </c>
       <c r="G5" s="101"/>
       <c r="H5" s="145"/>
       <c r="I5" s="123">
         <f>IF(B5="SI",IF($D5="SI",($F5+$G5+$H5) / (1- SUM($D$16:$D$20)),$F5),0)</f>
-        <v>0</v>
+        <v>1519.9143589743589</v>
       </c>
       <c r="J5" s="150">
         <f t="shared" ref="J5:J14" si="0">$K$3*$I5</f>
-        <v>0</v>
+        <v>133.3253676548718</v>
       </c>
     </row>
     <row r="6" spans="2:14" ht="19.95" customHeight="1" x14ac:dyDescent="0.35">
@@ -2592,26 +2593,26 @@
         <v>7</v>
       </c>
       <c r="E6" s="190">
-        <v>3.12</v>
+        <v>21.84</v>
       </c>
       <c r="F6" s="102">
         <f>E6*$F$2</f>
-        <v>3.12</v>
+        <v>43.68</v>
       </c>
       <c r="G6" s="101"/>
       <c r="H6" s="145"/>
       <c r="I6" s="123">
         <f t="shared" ref="I6:I14" si="1">IF(B6="SI",IF($D6="SI",($F6+$G6+$H6) / (1- SUM($D$16:$D$20)),$F6),0)</f>
-        <v>3.12</v>
+        <v>43.68</v>
       </c>
       <c r="J6" s="150">
         <f t="shared" si="0"/>
-        <v>0.27368328000000003</v>
+        <v>3.8315659200000001</v>
       </c>
     </row>
     <row r="7" spans="2:14" ht="19.95" customHeight="1" x14ac:dyDescent="0.35">
       <c r="B7" s="89" t="s">
-        <v>6</v>
+        <v>7</v>
       </c>
       <c r="C7" s="46" t="s">
         <v>11</v>
@@ -2624,17 +2625,17 @@
       </c>
       <c r="F7" s="102">
         <f t="shared" ref="F7:F11" si="2">E7*$F$2</f>
-        <v>3.6</v>
+        <v>7.2</v>
       </c>
       <c r="G7" s="103"/>
       <c r="H7" s="146"/>
       <c r="I7" s="123">
         <f t="shared" si="1"/>
-        <v>3.6</v>
+        <v>0</v>
       </c>
       <c r="J7" s="150">
         <f t="shared" si="0"/>
-        <v>0.31578840000000002</v>
+        <v>0</v>
       </c>
     </row>
     <row r="8" spans="2:14" ht="19.95" customHeight="1" x14ac:dyDescent="0.35">
@@ -2676,21 +2677,21 @@
         <v>7</v>
       </c>
       <c r="E9" s="190">
-        <v>7.8</v>
+        <v>54.6</v>
       </c>
       <c r="F9" s="102">
         <f t="shared" si="2"/>
-        <v>7.8</v>
+        <v>109.2</v>
       </c>
       <c r="G9" s="103"/>
       <c r="H9" s="146"/>
       <c r="I9" s="123">
         <f t="shared" si="1"/>
-        <v>7.8</v>
+        <v>109.2</v>
       </c>
       <c r="J9" s="150">
         <f t="shared" si="0"/>
-        <v>0.68420820000000004</v>
+        <v>9.5789148000000015</v>
       </c>
     </row>
     <row r="10" spans="2:14" ht="19.95" customHeight="1" x14ac:dyDescent="0.35">
@@ -2704,21 +2705,21 @@
         <v>7</v>
       </c>
       <c r="E10" s="190">
-        <v>7.92</v>
+        <v>80.64</v>
       </c>
       <c r="F10" s="102">
         <f t="shared" si="2"/>
-        <v>7.92</v>
+        <v>161.28</v>
       </c>
       <c r="G10" s="103"/>
       <c r="H10" s="146"/>
       <c r="I10" s="123">
         <f t="shared" si="1"/>
-        <v>7.92</v>
+        <v>161.28</v>
       </c>
       <c r="J10" s="150">
         <f t="shared" si="0"/>
-        <v>0.69473448000000004</v>
+        <v>14.14732032</v>
       </c>
     </row>
     <row r="11" spans="2:14" ht="19.95" customHeight="1" x14ac:dyDescent="0.35">
@@ -2732,21 +2733,21 @@
         <v>7</v>
       </c>
       <c r="E11" s="190">
-        <v>6.34</v>
+        <v>44.377200000000002</v>
       </c>
       <c r="F11" s="102">
         <f t="shared" si="2"/>
-        <v>6.34</v>
+        <v>88.754400000000004</v>
       </c>
       <c r="G11" s="103"/>
       <c r="H11" s="146"/>
       <c r="I11" s="123">
         <f t="shared" si="1"/>
-        <v>6.34</v>
+        <v>88.754400000000004</v>
       </c>
       <c r="J11" s="150">
         <f t="shared" si="0"/>
-        <v>0.55613846</v>
+        <v>7.7854472136000012</v>
       </c>
     </row>
     <row r="12" spans="2:14" ht="19.95" customHeight="1" x14ac:dyDescent="0.35">
@@ -2822,17 +2823,17 @@
       <c r="E15" s="141"/>
       <c r="F15" s="142">
         <f>SUM(F4:F14)</f>
-        <v>649.69288999999992</v>
+        <v>6803.3255999999992</v>
       </c>
       <c r="G15" s="143"/>
       <c r="H15" s="139"/>
       <c r="I15" s="152">
         <f>SUM(I4:I14)</f>
-        <v>824.82216666666659</v>
+        <v>8599.3390153846158</v>
       </c>
       <c r="J15" s="124">
         <f>SUM(J4:J14)</f>
-        <v>72.352575637833326</v>
+        <v>754.32541909052304</v>
       </c>
     </row>
     <row r="16" spans="2:14" ht="18" x14ac:dyDescent="0.35">
@@ -2851,11 +2852,11 @@
       <c r="H16" s="93"/>
       <c r="I16" s="120">
         <f>$I$4*$D16</f>
-        <v>119.40632499999998</v>
+        <v>1001.4765384615384</v>
       </c>
       <c r="J16" s="22">
         <f>$J$4*$D16</f>
-        <v>10.474203422674998</v>
+        <v>87.848520477307687</v>
       </c>
     </row>
     <row r="17" spans="2:10" ht="18" x14ac:dyDescent="0.35">
@@ -2872,11 +2873,11 @@
       <c r="H17" s="26"/>
       <c r="I17" s="119">
         <f>$I$4*$D17</f>
-        <v>39.802108333333337</v>
+        <v>333.82551282051281</v>
       </c>
       <c r="J17" s="24">
         <f t="shared" ref="J17:J20" si="3">$J$4*$D17</f>
-        <v>3.4914011408916665</v>
+        <v>29.282840159102562</v>
       </c>
     </row>
     <row r="18" spans="2:10" ht="18" x14ac:dyDescent="0.35">
@@ -2893,11 +2894,11 @@
       <c r="H18" s="26"/>
       <c r="I18" s="119">
         <f>$I$4*$D18</f>
-        <v>7.9604216666666661</v>
+        <v>66.765102564102563</v>
       </c>
       <c r="J18" s="24">
         <f t="shared" si="3"/>
-        <v>0.69828022817833335</v>
+        <v>5.8565680318205127</v>
       </c>
     </row>
     <row r="19" spans="2:10" ht="18" x14ac:dyDescent="0.35">
@@ -2914,11 +2915,11 @@
       <c r="H19" s="26"/>
       <c r="I19" s="119">
         <f>$I$4*$D19</f>
-        <v>7.9604216666666661</v>
+        <v>66.765102564102563</v>
       </c>
       <c r="J19" s="24">
         <f t="shared" si="3"/>
-        <v>0.69828022817833335</v>
+        <v>5.8565680318205127</v>
       </c>
     </row>
     <row r="20" spans="2:10" ht="18.600000000000001" thickBot="1" x14ac:dyDescent="0.4">
@@ -2952,11 +2953,11 @@
       <c r="H21" s="136"/>
       <c r="I21" s="137">
         <f>I15/(1-$D$22)</f>
-        <v>1031.0277083333331</v>
+        <v>10749.173769230769</v>
       </c>
       <c r="J21" s="125">
         <f>J15/(1-$D$22)</f>
-        <v>90.44071954729165</v>
+        <v>942.90677386315372</v>
       </c>
     </row>
     <row r="22" spans="2:10" ht="18.600000000000001" thickBot="1" x14ac:dyDescent="0.4">
@@ -2972,11 +2973,11 @@
       <c r="H22" s="20"/>
       <c r="I22" s="120">
         <f>$I$21*$D22</f>
-        <v>206.20554166666662</v>
+        <v>2149.8347538461539</v>
       </c>
       <c r="J22" s="128">
         <f>$J$21*$D22</f>
-        <v>18.088143909458331</v>
+        <v>188.58135477263076</v>
       </c>
     </row>
     <row r="23" spans="2:10" ht="18.600000000000001" thickBot="1" x14ac:dyDescent="0.35">
@@ -2994,7 +2995,7 @@
         <v>5</v>
       </c>
       <c r="D24" s="111">
-        <v>0.02</v>
+        <v>1.4800000000000001E-2</v>
       </c>
       <c r="E24" s="178"/>
       <c r="F24" s="8"/>
@@ -3002,11 +3003,11 @@
       <c r="H24" s="8"/>
       <c r="I24" s="122">
         <f>$I$28*$D24</f>
-        <v>25.775692708333327</v>
+        <v>214.78059479574753</v>
       </c>
       <c r="J24" s="22">
         <f>$J$28*$D24</f>
-        <v>2.261017988682291</v>
+        <v>18.840338994888175</v>
       </c>
     </row>
     <row r="25" spans="2:10" ht="18" x14ac:dyDescent="0.35">
@@ -3014,7 +3015,7 @@
         <v>26</v>
       </c>
       <c r="D25" s="35">
-        <v>0.02</v>
+        <v>8.4501000000000007E-2</v>
       </c>
       <c r="E25" s="176"/>
       <c r="F25" s="9"/>
@@ -3022,11 +3023,11 @@
       <c r="H25" s="9"/>
       <c r="I25" s="119">
         <f>$I$28*$D25</f>
-        <v>25.775692708333327</v>
+        <v>1226.2956108672608</v>
       </c>
       <c r="J25" s="24">
         <f t="shared" ref="J25:J27" si="4">$J$28*$D25</f>
-        <v>2.261017988682291</v>
+        <v>107.56942468966524</v>
       </c>
     </row>
     <row r="26" spans="2:10" ht="18" x14ac:dyDescent="0.35">
@@ -3042,11 +3043,11 @@
       <c r="H26" s="40"/>
       <c r="I26" s="119">
         <f>$I$28*$D26</f>
-        <v>38.663539062499986</v>
+        <v>435.36607053192063</v>
       </c>
       <c r="J26" s="24">
         <f t="shared" si="4"/>
-        <v>3.3915269830234367</v>
+        <v>38.189876340989535</v>
       </c>
     </row>
     <row r="27" spans="2:10" ht="18.600000000000001" thickBot="1" x14ac:dyDescent="0.4">
@@ -3062,11 +3063,11 @@
       <c r="H27" s="25"/>
       <c r="I27" s="119">
         <f>$I$28*$D27</f>
-        <v>167.54200260416664</v>
+        <v>1886.5863056383228</v>
       </c>
       <c r="J27" s="24">
         <f t="shared" si="4"/>
-        <v>14.696616926434892</v>
+        <v>165.48946414428801</v>
       </c>
     </row>
     <row r="28" spans="2:10" ht="18.600000000000001" thickBot="1" x14ac:dyDescent="0.35">
@@ -3080,11 +3081,11 @@
       <c r="H28" s="187"/>
       <c r="I28" s="152">
         <f>I21/(1-SUM($D$24:$D$27))</f>
-        <v>1288.7846354166663</v>
+        <v>14512.202351064021</v>
       </c>
       <c r="J28" s="188">
         <f>J21/(1-SUM($D$24:$D$27))</f>
-        <v>113.05089943411456</v>
+        <v>1272.9958780329846</v>
       </c>
     </row>
   </sheetData>

</xml_diff>